<commit_message>
Portals, routes, templates, seed, run.py and pytest suite
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/losses.xlsx
+++ b/sample_data/losses.xlsx
@@ -784,11 +784,7 @@
           <t>Test series no.</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>CPRIBLRSCL25T1654</t>
-        </is>
-      </c>
+      <c r="C6" s="6" t="n"/>
       <c r="D6" s="7" t="n"/>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
@@ -799,11 +795,7 @@
           <t>CPRI sample code</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>HVD25S0847</t>
-        </is>
-      </c>
+      <c r="C7" s="6" t="n"/>
       <c r="D7" s="7" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>

</xml_diff>